<commit_message>
Ajustar dashboard COLMED 2026 con filtros de fecha y provisiones diarias
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/odoo/cuotas_2026_01.xlsx
+++ b/odoo/cuotas_2026_01.xlsx
@@ -5404,7 +5404,7 @@
     <t>JONATHAN ALEXIS PÉREZ</t>
   </si>
   <si>
-    <t xml:space="preserve">ENA LISSETTE MERLOS </t>
+    <t>ENA LISSETTE MERLOS DE MIRANDA</t>
   </si>
   <si>
     <t>JAIME MAURICIO CASTRO AVALOS</t>
@@ -14738,7 +14738,7 @@
         <v>1264</v>
       </c>
       <c r="J260" s="3" t="s">
-        <v>969</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="261" spans="1:10">
@@ -24594,7 +24594,7 @@
         <v>1526</v>
       </c>
       <c r="J568" s="3" t="s">
-        <v>1998</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="569" spans="1:10">
@@ -32050,7 +32050,7 @@
         <v>1655</v>
       </c>
       <c r="J801" s="3" t="s">
-        <v>969</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="802" spans="1:10">
@@ -32082,7 +32082,7 @@
         <v>1655</v>
       </c>
       <c r="J802" s="3" t="s">
-        <v>969</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="803" spans="1:10">
@@ -32114,7 +32114,7 @@
         <v>1655</v>
       </c>
       <c r="J803" s="3" t="s">
-        <v>969</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="804" spans="1:10">
@@ -32146,7 +32146,7 @@
         <v>1655</v>
       </c>
       <c r="J804" s="3" t="s">
-        <v>969</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="805" spans="1:10">
@@ -32178,7 +32178,7 @@
         <v>1655</v>
       </c>
       <c r="J805" s="3" t="s">
-        <v>969</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="806" spans="1:10">
@@ -32210,7 +32210,7 @@
         <v>1655</v>
       </c>
       <c r="J806" s="3" t="s">
-        <v>969</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="807" spans="1:10">
@@ -33490,7 +33490,7 @@
         <v>1655</v>
       </c>
       <c r="J846" s="3" t="s">
-        <v>969</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="847" spans="1:10">
@@ -33522,7 +33522,7 @@
         <v>1655</v>
       </c>
       <c r="J847" s="3" t="s">
-        <v>969</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="848" spans="1:10">
@@ -33554,7 +33554,7 @@
         <v>1655</v>
       </c>
       <c r="J848" s="3" t="s">
-        <v>969</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="849" spans="1:10">
@@ -36946,7 +36946,7 @@
         <v>1714</v>
       </c>
       <c r="J954" s="3" t="s">
-        <v>1998</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="955" spans="1:10">
@@ -36978,7 +36978,7 @@
         <v>1714</v>
       </c>
       <c r="J955" s="3" t="s">
-        <v>1998</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="956" spans="1:10">
@@ -37010,7 +37010,7 @@
         <v>1714</v>
       </c>
       <c r="J956" s="3" t="s">
-        <v>1998</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="957" spans="1:10">
@@ -37042,7 +37042,7 @@
         <v>1714</v>
       </c>
       <c r="J957" s="3" t="s">
-        <v>1998</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="958" spans="1:10">
@@ -37074,7 +37074,7 @@
         <v>1714</v>
       </c>
       <c r="J958" s="3" t="s">
-        <v>1998</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="959" spans="1:10">
@@ -37106,7 +37106,7 @@
         <v>1714</v>
       </c>
       <c r="J959" s="3" t="s">
-        <v>1998</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="960" spans="1:10">
@@ -37138,7 +37138,7 @@
         <v>1714</v>
       </c>
       <c r="J960" s="3" t="s">
-        <v>1998</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="961" spans="1:10">
@@ -37170,7 +37170,7 @@
         <v>1714</v>
       </c>
       <c r="J961" s="3" t="s">
-        <v>1998</v>
+        <v>2002</v>
       </c>
     </row>
     <row r="962" spans="1:10">
@@ -49196,7 +49196,7 @@
         <v>1903</v>
       </c>
       <c r="J1337" s="3" t="s">
-        <v>1998</v>
+        <v>2001</v>
       </c>
     </row>
     <row r="1338" spans="1:10">
@@ -59948,7 +59948,7 @@
         <v>1264</v>
       </c>
       <c r="J1673" s="3" t="s">
-        <v>969</v>
+        <v>1998</v>
       </c>
     </row>
     <row r="1674" spans="1:10">

</xml_diff>